<commit_message>
ajout compétence du projet android
</commit_message>
<xml_diff>
--- a/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
+++ b/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cbc9f0bb248b3f74/Bureau/siteanais/Portfolio/t_competences/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{34F75D9C-4FAB-4279-B9B4-691CBE1EE43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7003BAC7-ED3C-4028-8352-930453307BBC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D272D328-B155-44A2-9186-A6E0C3A4D178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1125" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -230,6 +230,15 @@
   </si>
   <si>
     <t>▸Mettre en œuvre des outils et des stratégies de veille informationnelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet Android </t>
+  </si>
+  <si>
+    <t>03/11/2025 au 15/12/2025</t>
+  </si>
+  <si>
+    <t>▸Analyser les objectifs et les modalités d’organisation d’un projet</t>
   </si>
 </sst>
 </file>
@@ -363,7 +372,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -653,6 +662,58 @@
       </right>
       <top style="thin">
         <color rgb="FF4A452A"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF4A452A"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF4A452A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4A452A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF4A452A"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF4A452A"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF4A452A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
@@ -665,7 +726,7 @@
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -767,6 +828,30 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -776,29 +861,38 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1191,7 +1285,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ25"/>
+  <dimension ref="A1:AQ26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75.109375" style="1" customWidth="1"/>
@@ -1208,56 +1302,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35" t="s">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="35"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37" t="s">
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="2" t="s">
         <v>34</v>
       </c>
@@ -1269,22 +1363,22 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
     </row>
     <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="41" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -1307,8 +1401,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="8" customFormat="1" ht="324.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="42"/>
-      <c r="B7" s="43"/>
+      <c r="A7" s="40"/>
+      <c r="B7" s="41"/>
       <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
@@ -1329,14 +1423,14 @@
       </c>
     </row>
     <row r="8" spans="1:13" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
+      <c r="A8" s="42"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
     </row>
     <row r="9" spans="1:13" s="8" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
@@ -1431,91 +1525,97 @@
       <c r="B14" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="20"/>
+      <c r="C14" s="49"/>
       <c r="D14" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23" t="s">
+      <c r="E14" s="49"/>
+      <c r="F14" s="50"/>
+      <c r="G14" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="H14" s="21"/>
-    </row>
-    <row r="15" spans="1:13" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A15" s="38" t="s">
+      <c r="H14" s="51"/>
+    </row>
+    <row r="15" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="52"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="56" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="53"/>
+      <c r="H15" s="55"/>
+    </row>
+    <row r="16" spans="1:13" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A16" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="38"/>
-      <c r="H15" s="38"/>
-    </row>
-    <row r="16" spans="1:13" s="8" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="26" t="s">
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="47"/>
+    </row>
+    <row r="17" spans="1:9" s="8" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B17" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23" t="s">
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="22" t="s">
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="I16" s="28" t="s">
+      <c r="I17" s="28" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="8" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+    <row r="18" spans="1:9" s="8" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A18" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-    </row>
-    <row r="18" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+    </row>
+    <row r="19" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="45" t="s">
+      <c r="B19" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="23" t="s">
+      <c r="C19" s="11"/>
+      <c r="D19" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="22" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
-      <c r="H19" s="16"/>
-    </row>
-    <row r="20" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H19" s="22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="B20" s="10"/>
       <c r="C20" s="11"/>
@@ -1525,7 +1625,7 @@
       <c r="G20" s="11"/>
       <c r="H20" s="16"/>
     </row>
-    <row r="21" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="10"/>
       <c r="C21" s="11"/>
@@ -1535,7 +1635,7 @@
       <c r="G21" s="11"/>
       <c r="H21" s="16"/>
     </row>
-    <row r="22" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="10"/>
       <c r="C22" s="11"/>
@@ -1545,7 +1645,7 @@
       <c r="G22" s="11"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
       <c r="B23" s="10"/>
       <c r="C23" s="11"/>
@@ -1555,40 +1655,50 @@
       <c r="G23" s="11"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="18"/>
-    </row>
-    <row r="25" spans="1:8" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
+    <row r="24" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="16"/>
+    </row>
+    <row r="25" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="18"/>
+    </row>
+    <row r="26" spans="1:9" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A26" s="13"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ajout du projet moderation avec iteration1
</commit_message>
<xml_diff>
--- a/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
+++ b/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cbc9f0bb248b3f74/Bureau/siteanais/Portfolio/t_competences/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D272D328-B155-44A2-9186-A6E0C3A4D178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEFA4962-8670-4CA2-B6D0-37DB6851958F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1125" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
@@ -28,12 +28,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
-  </si>
-  <si>
-    <t>SESSION 2024</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
@@ -114,9 +111,6 @@
     <t>NOM et prénom : PORTOLLEAU Anaïs</t>
   </si>
   <si>
-    <t>Centre de formation : Joliverie</t>
-  </si>
-  <si>
     <t xml:space="preserve">08/01/2024 au 12/01/2024 </t>
   </si>
   <si>
@@ -130,9 +124,6 @@
   </si>
   <si>
     <t>13/05/2024 au 21/06/2024</t>
-  </si>
-  <si>
-    <t>Stage - 1ère année SIO à Orcab Artisans Artipole                                                  Application pour vérifier les urls/liens saisies par les coopératives dans DataSiteOrcab</t>
   </si>
   <si>
     <t xml:space="preserve">▸Collecter, suivre et orienter des demandes </t>
@@ -184,9 +175,6 @@
     <t>▸Participer à l’évolution d’un site Web exploitant les données de l’organisation.</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio :  https://anaisprt44.github.io/Portfolio/</t>
-  </si>
-  <si>
     <t>Projet Web - Intranet</t>
   </si>
   <si>
@@ -223,9 +211,6 @@
     <t>▸Mettre en place son environnement d’apprentissage personnel                                                                                                                                                ▸Gérer son identité professionnelle</t>
   </si>
   <si>
-    <t>Stage - 2nd année de BTS SIO à Delia Technologies - Applicationpour gérer</t>
-  </si>
-  <si>
     <t>05/01/26 au 12/02/26</t>
   </si>
   <si>
@@ -239,6 +224,38 @@
   </si>
   <si>
     <t>▸Analyser les objectifs et les modalités d’organisation d’un projet</t>
+  </si>
+  <si>
+    <t>SESSION 2026</t>
+  </si>
+  <si>
+    <t>Centre de formation : La Joliverie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pennylane </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stage - 2nd année de BTS SIO à Delia Technologies - Application web pour gérer les factures/transactions </t>
+  </si>
+  <si>
+    <t>Stage - 1ère année SIO à Orcab Artisans Artipole - Application pour vérifier les urls/liens saisies par les coopératives dans DataSiteOrcab</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Adresse URL du portfolio :  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://anaisprt44.github.io/Portfolio/</t>
+    </r>
+  </si>
+  <si>
+    <t>▸Déployer un service</t>
   </si>
 </sst>
 </file>
@@ -372,7 +389,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -604,51 +621,6 @@
         <color rgb="FF4A452A"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF4A452A"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF4A452A"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF4A452A"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF4A452A"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF4A452A"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF4A452A"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF4A452A"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF4A452A"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF4A452A"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF4A452A"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF4A452A"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF4A452A"/>
-      </top>
-      <bottom style="medium">
         <color rgb="FF4A452A"/>
       </bottom>
       <diagonal/>
@@ -726,7 +698,7 @@
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -752,18 +724,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -773,18 +736,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -802,9 +753,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -825,15 +773,54 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -852,47 +839,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1285,7 +1239,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ26"/>
+  <dimension ref="A1:AQ20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75.109375" style="1" customWidth="1"/>
@@ -1302,396 +1256,336 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="37"/>
+    </row>
+    <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="43"/>
-    </row>
-    <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+    </row>
+    <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-    </row>
-    <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+    </row>
+    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" s="8" customFormat="1" ht="324.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="45"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="47"/>
+      <c r="B8" s="47"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="47"/>
+    </row>
+    <row r="9" spans="1:13" s="8" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="15"/>
+    </row>
+    <row r="10" spans="1:13" s="8" customFormat="1" ht="97.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="2" t="s">
+      <c r="C10" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="16"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="15"/>
+    </row>
+    <row r="11" spans="1:13" s="8" customFormat="1" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="15"/>
+    </row>
+    <row r="12" spans="1:13" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="G12" s="13"/>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:13" s="8" customFormat="1" ht="73.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-    </row>
-    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="40" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" s="8" customFormat="1" ht="324.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="40"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="7" t="s">
+      <c r="B13" s="26"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="29"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="H14" s="31"/>
+    </row>
+    <row r="15" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="32"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="33"/>
+      <c r="H15" s="35"/>
+    </row>
+    <row r="16" spans="1:13" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A16" s="40" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="42"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-    </row>
-    <row r="9" spans="1:13" s="8" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
+    </row>
+    <row r="17" spans="1:9" s="8" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="I17" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="22"/>
-    </row>
-    <row r="10" spans="1:13" s="8" customFormat="1" ht="97.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="22"/>
-    </row>
-    <row r="11" spans="1:13" s="8" customFormat="1" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="22"/>
-    </row>
-    <row r="12" spans="1:13" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="20"/>
-      <c r="H12" s="21"/>
-    </row>
-    <row r="13" spans="1:13" s="8" customFormat="1" ht="73.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="34"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="22" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="25" t="s">
+    </row>
+    <row r="18" spans="1:9" s="8" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A18" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+    </row>
+    <row r="19" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="50" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="49"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="50" t="s">
+      <c r="C19" s="9"/>
+      <c r="D19" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H14" s="51"/>
-    </row>
-    <row r="15" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="46" t="s">
+      <c r="I19" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="48" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="G15" s="53"/>
-      <c r="H15" s="55"/>
-    </row>
-    <row r="16" spans="1:13" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A16" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
-    </row>
-    <row r="17" spans="1:9" s="8" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="I17" s="28" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" s="8" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-    </row>
-    <row r="19" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="22" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="16"/>
-    </row>
-    <row r="21" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="16"/>
-    </row>
-    <row r="22" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="16"/>
-    </row>
-    <row r="23" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="16"/>
-    </row>
-    <row r="24" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="16"/>
-    </row>
-    <row r="25" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
-    </row>
-    <row r="26" spans="1:9" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
+    </row>
+    <row r="20" spans="1:9" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A4:E4"/>
@@ -1699,6 +1593,11 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
mise à jour des veilles +  début du projet modération
</commit_message>
<xml_diff>
--- a/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
+++ b/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cbc9f0bb248b3f74/Bureau/siteanais/Portfolio/t_competences/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEFA4962-8670-4CA2-B6D0-37DB6851958F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{CEFA4962-8670-4CA2-B6D0-37DB6851958F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23043BE9-0DDE-4C93-842E-8DB0E00FAE6F}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14775" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$21</definedName>
   </definedNames>
   <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -241,9 +241,18 @@
     <t>Stage - 1ère année SIO à Orcab Artisans Artipole - Application pour vérifier les urls/liens saisies par les coopératives dans DataSiteOrcab</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Adresse URL du portfolio :  </t>
-    </r>
+    <t>▸Déployer un service</t>
+  </si>
+  <si>
+    <t>09/03/2026 au 30/03/2026</t>
+  </si>
+  <si>
+    <t>Projet Java - Application de modération du site R3st0.fr</t>
+  </si>
+  <si>
+    <t>Déployer un service</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -251,11 +260,19 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">Adresse URL du portfolio :  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="18"/>
+        <color theme="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t>https://anaisprt44.github.io/Portfolio/</t>
     </r>
-  </si>
-  <si>
-    <t>▸Déployer un service</t>
   </si>
 </sst>
 </file>
@@ -265,7 +282,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* \-??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -321,12 +338,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="16"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -347,12 +358,6 @@
       <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -368,14 +373,41 @@
       <family val="2"/>
     </font>
     <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <u/>
-      <sz val="10"/>
+      <sz val="18"/>
       <color theme="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -695,10 +727,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -724,87 +756,102 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -815,21 +862,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -839,14 +883,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1239,7 +1277,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ20"/>
+  <dimension ref="A1:AQ21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75.109375" style="1" customWidth="1"/>
@@ -1256,83 +1294,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37" t="s">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="37"/>
+      <c r="H1" s="42"/>
     </row>
     <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="39" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="39"/>
-      <c r="H3" s="39"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
       <c r="F4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="H4" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
+      <c r="A5" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
     </row>
     <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="50" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -1355,8 +1393,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="8" customFormat="1" ht="324.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="45"/>
-      <c r="B7" s="46"/>
+      <c r="A7" s="49"/>
+      <c r="B7" s="50"/>
       <c r="C7" s="6" t="s">
         <v>12</v>
       </c>
@@ -1377,217 +1415,245 @@
       </c>
     </row>
     <row r="8" spans="1:13" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
+      <c r="A8" s="51"/>
+      <c r="B8" s="51"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="51"/>
     </row>
     <row r="9" spans="1:13" s="8" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="32"/>
     </row>
     <row r="10" spans="1:13" s="8" customFormat="1" ht="97.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="16"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="32"/>
     </row>
     <row r="11" spans="1:13" s="8" customFormat="1" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="32"/>
     </row>
     <row r="12" spans="1:13" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13" t="s">
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="14"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="32"/>
     </row>
     <row r="13" spans="1:13" s="8" customFormat="1" ht="73.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13" t="s">
+      <c r="B13" s="34"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" s="32"/>
+    </row>
+    <row r="14" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="22"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="H14" s="24"/>
+      <c r="I14" s="32"/>
+    </row>
+    <row r="15" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="25"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="26"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="32"/>
+    </row>
+    <row r="16" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="25" t="s">
+      <c r="C16" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="27"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" s="28"/>
+      <c r="I16" s="32"/>
+    </row>
+    <row r="17" spans="1:9" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A17" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="32"/>
+    </row>
+    <row r="18" spans="1:9" s="8" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I18" s="38" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="8" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A19" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="32"/>
+    </row>
+    <row r="20" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="40"/>
+      <c r="D20" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="29"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="H14" s="31"/>
-    </row>
-    <row r="15" spans="1:13" s="8" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="32"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="G15" s="33"/>
-      <c r="H15" s="35"/>
-    </row>
-    <row r="16" spans="1:13" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A16" s="40" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="41"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
-    </row>
-    <row r="17" spans="1:9" s="8" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="49" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="I17" s="20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" s="8" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A18" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="42"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-    </row>
-    <row r="19" spans="1:9" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="50" t="s">
-        <v>56</v>
-      </c>
-      <c r="B19" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="15" t="s">
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="I20" s="32" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
+    <row r="21" spans="1:9" s="8" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A6:A7"/>
@@ -1599,8 +1665,11 @@
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="F3:H3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A5:H5" r:id="rId1" display="Adresse URL du portfolio :  https://anaisprt44.github.io/Portfolio/" xr:uid="{73D7E004-B80F-41DA-A367-A5252A13D356}"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
mise à jour des compétences
</commit_message>
<xml_diff>
--- a/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
+++ b/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anais\Downloads\Epreuve_E5\Portfolio\t_competences\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0764629B-961F-4D65-A95B-E772926F9A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE5E0FE7-A133-4689-80B0-393156E5DF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14775" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -163,9 +163,6 @@
     <t>▸Gérer des sauvegardes</t>
   </si>
   <si>
-    <t xml:space="preserve">▸Recenser et identifier les ressources numériques                                        ▸Mettre en place et vérifier les niveaux d’habilitation associés à un service                                                                              </t>
-  </si>
-  <si>
     <t>15/09/2025 au 13/10/2025</t>
   </si>
   <si>
@@ -212,9 +209,6 @@
   </si>
   <si>
     <t>Projet Java - Application de modération du site R3st0.fr</t>
-  </si>
-  <si>
-    <t>Déployer un service</t>
   </si>
   <si>
     <r>
@@ -272,6 +266,15 @@
       </rPr>
       <t>https://anaisprt44.github.io/Portfolio/index.html</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">▸Gérer des sauvegardes    ▸Recenser et identifier les ressources numériques  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">▸ Déployer un service ▸Accompagner les utilisateurs dans la mise en place d’un service </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ▸Mettre en place et vérifier les niveaux d’habilitation associés à un service                                                                              </t>
   </si>
 </sst>
 </file>
@@ -904,6 +907,30 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -957,30 +984,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1391,28 +1394,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:1296" x14ac:dyDescent="0.25">
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
     </row>
     <row r="2" spans="2:1296" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60" t="s">
-        <v>49</v>
-      </c>
-      <c r="I2" s="60"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" s="42"/>
       <c r="J2" s="9"/>
       <c r="L2"/>
       <c r="M2"/>
@@ -2701,41 +2704,41 @@
       <c r="AWV2"/>
     </row>
     <row r="3" spans="2:1296" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:1296" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="65" t="s">
-        <v>59</v>
-      </c>
-      <c r="H4" s="63"/>
-      <c r="I4" s="66"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" s="45"/>
+      <c r="I4" s="48"/>
       <c r="J4" s="9"/>
     </row>
     <row r="5" spans="2:1296" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="46" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="48"/>
+      <c r="B5" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="56"/>
       <c r="G5" s="5" t="s">
         <v>29</v>
       </c>
@@ -2743,28 +2746,28 @@
         <v>2</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J5" s="9"/>
     </row>
     <row r="6" spans="2:1296" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="49" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="51"/>
+      <c r="B6" s="57" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="59"/>
       <c r="J6" s="9"/>
     </row>
     <row r="7" spans="2:1296" ht="91.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="52" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="54" t="s">
+      <c r="B7" s="60" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" s="62" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="32" t="s">
@@ -2788,8 +2791,8 @@
       <c r="J7" s="9"/>
     </row>
     <row r="8" spans="2:1296" s="3" customFormat="1" ht="196.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="53"/>
-      <c r="C8" s="55"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="63"/>
       <c r="D8" s="7" t="s">
         <v>10</v>
       </c>
@@ -2812,14 +2815,14 @@
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="2:1296" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="56"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="57"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="58"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
+      <c r="I9" s="66"/>
       <c r="J9" s="9"/>
       <c r="K9" s="4"/>
     </row>
@@ -2849,7 +2852,7 @@
         <v>20</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>24</v>
@@ -2863,7 +2866,7 @@
       <c r="J11" s="14"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="2:1296" s="3" customFormat="1" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:1296" s="3" customFormat="1" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
         <v>22</v>
       </c>
@@ -2891,9 +2894,11 @@
         <v>34</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>63</v>
+      </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13" t="s">
         <v>31</v>
@@ -2913,20 +2918,20 @@
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J14" s="14"/>
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="2:1296" s="3" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" s="39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D15" s="18"/>
       <c r="E15" s="19" t="s">
@@ -2935,7 +2940,7 @@
       <c r="F15" s="18"/>
       <c r="G15" s="20"/>
       <c r="H15" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I15" s="21"/>
       <c r="J15" s="14"/>
@@ -2943,16 +2948,16 @@
     </row>
     <row r="16" spans="2:1296" s="3" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="40" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="40" t="s">
-        <v>47</v>
       </c>
       <c r="D16" s="23"/>
       <c r="E16" s="24"/>
       <c r="F16" s="25"/>
       <c r="G16" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H16" s="27"/>
       <c r="I16" s="25"/>
@@ -2961,10 +2966,10 @@
     </row>
     <row r="17" spans="1:11" s="3" customFormat="1" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D17" s="28" t="s">
         <v>38</v>
@@ -2973,29 +2978,29 @@
       <c r="F17" s="25"/>
       <c r="G17" s="26"/>
       <c r="H17" s="27" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I17" s="25"/>
       <c r="J17" s="14"/>
       <c r="K17" s="4"/>
     </row>
     <row r="18" spans="1:11" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
       <c r="J18" s="14"/>
       <c r="K18" s="4"/>
     </row>
     <row r="19" spans="1:11" s="3" customFormat="1" ht="109.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="15" t="s">
         <v>23</v>
@@ -3008,7 +3013,7 @@
       <c r="G19" s="30"/>
       <c r="H19" s="30"/>
       <c r="I19" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J19" s="14" t="s">
         <v>28</v>
@@ -3016,25 +3021,25 @@
       <c r="K19" s="4"/>
     </row>
     <row r="20" spans="1:11" s="3" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B20" s="43" t="s">
+      <c r="B20" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="45"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="53"/>
       <c r="J20" s="14"/>
       <c r="K20" s="4"/>
     </row>
     <row r="21" spans="1:11" s="3" customFormat="1" ht="82.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21" s="35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D21" s="31"/>
       <c r="E21" s="10" t="s">
@@ -3044,10 +3049,10 @@
       <c r="G21" s="31"/>
       <c r="H21" s="31"/>
       <c r="I21" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K21" s="4"/>
     </row>
@@ -3174,12 +3179,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G4:I4"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="B5:F5"/>
@@ -3187,6 +3186,12 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G4:I4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B6:I6" r:id="rId1" display="Adresse URL du portfolio :  https://anaisprt44.github.io/Portfolio/" xr:uid="{73D7E004-B80F-41DA-A367-A5252A13D356}"/>

</xml_diff>

<commit_message>
mise à jour du tableau de compétences
</commit_message>
<xml_diff>
--- a/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
+++ b/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anais\Downloads\Epreuve_E5\Portfolio\t_competences\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE5E0FE7-A133-4689-80B0-393156E5DF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543B5352-C300-4092-ABA1-DA99550692A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="64">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -907,6 +907,60 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -930,60 +984,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1394,28 +1394,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:1296" x14ac:dyDescent="0.25">
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
     </row>
     <row r="2" spans="2:1296" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42" t="s">
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="42"/>
+      <c r="I2" s="60"/>
       <c r="J2" s="9"/>
       <c r="L2"/>
       <c r="M2"/>
@@ -2704,41 +2704,41 @@
       <c r="AWV2"/>
     </row>
     <row r="3" spans="2:1296" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:1296" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="47" t="s">
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="45"/>
-      <c r="I4" s="48"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="66"/>
       <c r="J4" s="9"/>
     </row>
     <row r="5" spans="2:1296" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="56"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="48"/>
       <c r="G5" s="5" t="s">
         <v>29</v>
       </c>
@@ -2751,23 +2751,23 @@
       <c r="J5" s="9"/>
     </row>
     <row r="6" spans="2:1296" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="58"/>
-      <c r="I6" s="59"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="50"/>
+      <c r="G6" s="50"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="51"/>
       <c r="J6" s="9"/>
     </row>
     <row r="7" spans="2:1296" ht="91.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="52" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="62" t="s">
+      <c r="C7" s="54" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="32" t="s">
@@ -2791,8 +2791,8 @@
       <c r="J7" s="9"/>
     </row>
     <row r="8" spans="2:1296" s="3" customFormat="1" ht="196.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="61"/>
-      <c r="C8" s="63"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="55"/>
       <c r="D8" s="7" t="s">
         <v>10</v>
       </c>
@@ -2815,14 +2815,14 @@
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="2:1296" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="64"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="66"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="57"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="58"/>
       <c r="J9" s="9"/>
       <c r="K9" s="4"/>
     </row>
@@ -2896,9 +2896,7 @@
       <c r="D13" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>63</v>
-      </c>
+      <c r="E13" s="10"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13" t="s">
         <v>31</v>
@@ -2985,16 +2983,16 @@
       <c r="K17" s="4"/>
     </row>
     <row r="18" spans="1:11" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="49" t="s">
+      <c r="B18" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="50"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
       <c r="J18" s="14"/>
       <c r="K18" s="4"/>
     </row>
@@ -3021,16 +3019,16 @@
       <c r="K19" s="4"/>
     </row>
     <row r="20" spans="1:11" s="3" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B20" s="51" t="s">
+      <c r="B20" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="53"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="45"/>
       <c r="J20" s="14"/>
       <c r="K20" s="4"/>
     </row>
@@ -3179,6 +3177,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G4:I4"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="B5:F5"/>
@@ -3186,12 +3190,6 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G4:I4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B6:I6" r:id="rId1" display="Adresse URL du portfolio :  https://anaisprt44.github.io/Portfolio/" xr:uid="{73D7E004-B80F-41DA-A367-A5252A13D356}"/>

</xml_diff>

<commit_message>
correction de fautes + tableau
</commit_message>
<xml_diff>
--- a/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
+++ b/t_competences/Tableau de synthèse - BTS SIO 2024_PORTOLLEAU.xlsx
@@ -907,6 +907,30 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -960,30 +984,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1394,28 +1394,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:1296" x14ac:dyDescent="0.25">
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
     </row>
     <row r="2" spans="2:1296" ht="31.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="60"/>
+      <c r="I2" s="42"/>
       <c r="J2" s="9"/>
       <c r="L2"/>
       <c r="M2"/>
@@ -2704,41 +2704,41 @@
       <c r="AWV2"/>
     </row>
     <row r="3" spans="2:1296" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
       <c r="J3" s="9"/>
     </row>
     <row r="4" spans="2:1296" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="65" t="s">
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="63"/>
-      <c r="I4" s="66"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="48"/>
       <c r="J4" s="9"/>
     </row>
     <row r="5" spans="2:1296" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="48"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="56"/>
       <c r="G5" s="5" t="s">
         <v>29</v>
       </c>
@@ -2751,23 +2751,23 @@
       <c r="J5" s="9"/>
     </row>
     <row r="6" spans="2:1296" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="51"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="59"/>
       <c r="J6" s="9"/>
     </row>
     <row r="7" spans="2:1296" ht="91.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="52" t="s">
+      <c r="B7" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="62" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="32" t="s">
@@ -2791,8 +2791,8 @@
       <c r="J7" s="9"/>
     </row>
     <row r="8" spans="2:1296" s="3" customFormat="1" ht="196.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="53"/>
-      <c r="C8" s="55"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="63"/>
       <c r="D8" s="7" t="s">
         <v>10</v>
       </c>
@@ -2815,14 +2815,14 @@
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="2:1296" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="56"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="57"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="58"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
+      <c r="I9" s="66"/>
       <c r="J9" s="9"/>
       <c r="K9" s="4"/>
     </row>
@@ -2983,16 +2983,16 @@
       <c r="K17" s="4"/>
     </row>
     <row r="18" spans="1:11" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
       <c r="J18" s="14"/>
       <c r="K18" s="4"/>
     </row>
@@ -3019,16 +3019,16 @@
       <c r="K19" s="4"/>
     </row>
     <row r="20" spans="1:11" s="3" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B20" s="43" t="s">
+      <c r="B20" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="45"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="53"/>
       <c r="J20" s="14"/>
       <c r="K20" s="4"/>
     </row>
@@ -3177,12 +3177,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G4:I4"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B20:I20"/>
     <mergeCell ref="B5:F5"/>
@@ -3190,6 +3184,12 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G4:I4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B6:I6" r:id="rId1" display="Adresse URL du portfolio :  https://anaisprt44.github.io/Portfolio/" xr:uid="{73D7E004-B80F-41DA-A367-A5252A13D356}"/>

</xml_diff>